<commit_message>
Add lead logos to demos
</commit_message>
<xml_diff>
--- a/outputs/vitoria_saude_leads_20260605/leads_saude_vitoria_es_2026-06-05.xlsx
+++ b/outputs/vitoria_saude_leads_20260605/leads_saude_vitoria_es_2026-06-05.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" r:id="R8f203acc551445e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="2" r:id="Rd0b29fdcfd534a1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 3" sheetId="3" r:id="Rbca954b008654197"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" r:id="Re4850dfa1bbb4a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="2" r:id="R952528df64234701"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 3" sheetId="3" r:id="R42627360e1254593"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -728,28 +728,28 @@
         <x:v>&lt;=10 km</x:v>
       </x:c>
       <x:c r="G4" s="37" t="str">
-        <x:v>Portal/booking only</x:v>
+        <x:v>Google Sites + booking</x:v>
       </x:c>
       <x:c r="H4" s="37" t="str">
-        <x:v>Setmore + Instagram</x:v>
+        <x:v>Google Sites + Setmore + Instagram</x:v>
       </x:c>
       <x:c r="I4" s="37" t="str">
         <x:v>(27) 99779-6437</x:v>
       </x:c>
       <x:c r="J4" s="37" t="str">
-        <x:v>Usa agendamento externo, sem site próprio claro.</x:v>
+        <x:v>Tem site em Google Sites e agenda externa; oportunidade de melhorar presença própria.</x:v>
       </x:c>
       <x:c r="K4" s="37" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L4" s="37" t="str">
-        <x:v>https://centrodeterapiasintegrativasemsadeltda.setmore.com/</x:v>
+        <x:v>https://sites.google.com/view/essencesade</x:v>
       </x:c>
       <x:c r="M4" s="37" t="str">
-        <x:v>Fonte adicional: SindjudES lista Instagram e WhatsApp.</x:v>
+        <x:v>Fonte adicional: Setmore/SindjudES lista Instagram e WhatsApp.</x:v>
       </x:c>
       <x:c r="N4" s="38" t="str">
-        <x:v>Oferecer site leve integrado ao botão de reservas.</x:v>
+        <x:v>Oferecer redesign/landing page integrada ao WhatsApp e reservas.</x:v>
       </x:c>
       <x:c r="O4" s="1"/>
       <x:c r="P4" s="1"/>
@@ -6753,28 +6753,28 @@
   <x:sheetData>
     <x:row r="1" ht="31.5" customHeight="1">
       <x:c r="A1" s="49" t="str">
-        <x:v>Leads de saúde sem site próprio - Vitória/ES</x:v>
+        <x:v>Leads de saúde com presença digital fraca - Vitória/ES</x:v>
       </x:c>
       <x:c r="B1" s="50" t="str">
-        <x:v>Leads de saúde sem site próprio - Vitória/ES</x:v>
+        <x:v>Leads de saúde com presença digital fraca - Vitória/ES</x:v>
       </x:c>
       <x:c r="C1" s="50" t="str">
-        <x:v>Leads de saúde sem site próprio - Vitória/ES</x:v>
+        <x:v>Leads de saúde com presença digital fraca - Vitória/ES</x:v>
       </x:c>
       <x:c r="D1" s="50" t="str">
-        <x:v>Leads de saúde sem site próprio - Vitória/ES</x:v>
+        <x:v>Leads de saúde com presença digital fraca - Vitória/ES</x:v>
       </x:c>
       <x:c r="E1" s="50" t="str">
-        <x:v>Leads de saúde sem site próprio - Vitória/ES</x:v>
+        <x:v>Leads de saúde com presença digital fraca - Vitória/ES</x:v>
       </x:c>
       <x:c r="F1" s="50" t="str">
-        <x:v>Leads de saúde sem site próprio - Vitória/ES</x:v>
+        <x:v>Leads de saúde com presença digital fraca - Vitória/ES</x:v>
       </x:c>
       <x:c r="G1" s="50" t="str">
-        <x:v>Leads de saúde sem site próprio - Vitória/ES</x:v>
+        <x:v>Leads de saúde com presença digital fraca - Vitória/ES</x:v>
       </x:c>
       <x:c r="H1" s="51" t="str">
-        <x:v>Leads de saúde sem site próprio - Vitória/ES</x:v>
+        <x:v>Leads de saúde com presença digital fraca - Vitória/ES</x:v>
       </x:c>
       <x:c r="I1" s="1"/>
       <x:c r="J1" s="1"/>
@@ -6938,7 +6938,7 @@
         <x:v>Objetivo</x:v>
       </x:c>
       <x:c r="B6" s="38" t="str">
-        <x:v>Leads sem site próprio standalone</x:v>
+        <x:v>Leads sem site próprio forte ou dependentes de social/booking</x:v>
       </x:c>
       <x:c r="C6" s="1"/>
       <x:c r="D6" s="60" t="str">

</xml_diff>